<commit_message>
Update web favicon and adding all the medical of some teams.
</commit_message>
<xml_diff>
--- a/excel/player_employees.xlsx
+++ b/excel/player_employees.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="52">
   <si>
     <t>name</t>
   </si>
@@ -146,6 +146,27 @@
   </si>
   <si>
     <t>opm</t>
+  </si>
+  <si>
+    <t>Haruno Sakura</t>
+  </si>
+  <si>
+    <t>Medical</t>
+  </si>
+  <si>
+    <t>Yamanaka Ino</t>
+  </si>
+  <si>
+    <t>Tony Tony Chopper</t>
+  </si>
+  <si>
+    <t>Kocho Shinobu</t>
+  </si>
+  <si>
+    <t>Kocho Kanae</t>
+  </si>
+  <si>
+    <t>Kanzaki Aoi</t>
   </si>
 </sst>
 </file>
@@ -1622,40 +1643,88 @@
       </c>
     </row>
     <row r="22" ht="20.05" customHeight="1">
-      <c r="A22" s="7"/>
-      <c r="B22" s="7"/>
-      <c r="C22" s="7"/>
-      <c r="D22" s="7"/>
+      <c r="A22" t="s" s="5">
+        <v>45</v>
+      </c>
+      <c r="B22" s="6">
+        <v>35</v>
+      </c>
+      <c r="C22" t="s" s="5">
+        <v>46</v>
+      </c>
+      <c r="D22" t="s" s="5">
+        <v>10</v>
+      </c>
     </row>
     <row r="23" ht="20.05" customHeight="1">
-      <c r="A23" s="7"/>
-      <c r="B23" s="7"/>
-      <c r="C23" s="7"/>
-      <c r="D23" s="7"/>
+      <c r="A23" t="s" s="5">
+        <v>47</v>
+      </c>
+      <c r="B23" s="6">
+        <v>35</v>
+      </c>
+      <c r="C23" t="s" s="5">
+        <v>46</v>
+      </c>
+      <c r="D23" t="s" s="5">
+        <v>10</v>
+      </c>
     </row>
     <row r="24" ht="20.05" customHeight="1">
-      <c r="A24" s="7"/>
-      <c r="B24" s="7"/>
-      <c r="C24" s="7"/>
-      <c r="D24" s="7"/>
+      <c r="A24" t="s" s="5">
+        <v>48</v>
+      </c>
+      <c r="B24" s="6">
+        <v>24</v>
+      </c>
+      <c r="C24" t="s" s="5">
+        <v>46</v>
+      </c>
+      <c r="D24" t="s" s="5">
+        <v>30</v>
+      </c>
     </row>
     <row r="25" ht="20.05" customHeight="1">
-      <c r="A25" s="7"/>
-      <c r="B25" s="7"/>
-      <c r="C25" s="7"/>
-      <c r="D25" s="7"/>
+      <c r="A25" t="s" s="5">
+        <v>49</v>
+      </c>
+      <c r="B25" s="6">
+        <v>20</v>
+      </c>
+      <c r="C25" t="s" s="5">
+        <v>46</v>
+      </c>
+      <c r="D25" t="s" s="5">
+        <v>18</v>
+      </c>
     </row>
     <row r="26" ht="20.05" customHeight="1">
-      <c r="A26" s="7"/>
-      <c r="B26" s="7"/>
-      <c r="C26" s="7"/>
-      <c r="D26" s="7"/>
+      <c r="A26" t="s" s="5">
+        <v>50</v>
+      </c>
+      <c r="B26" s="6">
+        <v>22</v>
+      </c>
+      <c r="C26" t="s" s="5">
+        <v>46</v>
+      </c>
+      <c r="D26" t="s" s="5">
+        <v>18</v>
+      </c>
     </row>
     <row r="27" ht="20.05" customHeight="1">
-      <c r="A27" s="7"/>
-      <c r="B27" s="7"/>
-      <c r="C27" s="7"/>
-      <c r="D27" s="7"/>
+      <c r="A27" t="s" s="5">
+        <v>51</v>
+      </c>
+      <c r="B27" s="6">
+        <v>17</v>
+      </c>
+      <c r="C27" t="s" s="5">
+        <v>46</v>
+      </c>
+      <c r="D27" t="s" s="5">
+        <v>18</v>
+      </c>
     </row>
     <row r="28" ht="20.05" customHeight="1">
       <c r="A28" s="7"/>

</xml_diff>